<commit_message>
Add batch 3 Google Forms Qawwali registrations
</commit_message>
<xml_diff>
--- a/assets/Qawalli.xlsx
+++ b/assets/Qawalli.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Downloads\sentec-neduet-website-revised-main (1)\trewwws\sentec-pure-php\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{04C1ECF9-0086-4735-853C-999CD591358F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30D96C51-63BA-4595-B79F-5405549528DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,11 @@
     <sheet name="Form Responses 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t>Timestamp</t>
   </si>
@@ -44,73 +43,7 @@
     <t>University ( outside participant only)</t>
   </si>
   <si>
-    <t>Bcit</t>
-  </si>
-  <si>
-    <t>Ayesha qazi</t>
-  </si>
-  <si>
-    <t>03351025483</t>
-  </si>
-  <si>
-    <t>CT-26102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electrical Engineering </t>
-  </si>
-  <si>
-    <t>khizerr101@gmail.con</t>
-  </si>
-  <si>
-    <t>Muhammad Khizer</t>
-  </si>
-  <si>
-    <t>0332 7875503</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/open?id=1ECJE1XXp9iqKsrFMaGAjKUkw4NqlAJs1</t>
-  </si>
-  <si>
-    <t>EE-026</t>
-  </si>
-  <si>
-    <t>muneebsheikhh101@gmail.com</t>
-  </si>
-  <si>
-    <t>Muneeb Ahmed sheikh</t>
-  </si>
-  <si>
-    <t>0331 6713255</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/open?id=1wUPubYdOW8uj_38xDtH6iNZpVfET-Omy</t>
-  </si>
-  <si>
     <t>EE-017</t>
-  </si>
-  <si>
-    <t>muhammadhammadtariq189@gmail.com</t>
-  </si>
-  <si>
-    <t>Hammad Tariq</t>
-  </si>
-  <si>
-    <t>Muhammadhammadtariq189@gmail.com</t>
-  </si>
-  <si>
-    <t>03112813959</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/open?id=1ezdcL4FxXMNbKhhA9rrP1tZZcHXy_pn2</t>
-  </si>
-  <si>
-    <t>EE</t>
-  </si>
-  <si>
-    <t>rose77639126@gmail.com</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/open?id=1_ZpbENGA6ikoNn1XdsQ0EUOeRqJGXcGh</t>
   </si>
   <si>
     <t>email address2</t>
@@ -125,15 +58,87 @@
 Bank Name: Habib Metropolitan Bank Limited
 Bank Address: University Road Bran</t>
   </si>
+  <si>
+    <t>simrahhussain07@gmail.com</t>
+  </si>
+  <si>
+    <t>Simrah Hussain</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1VwWIqyBcA13SJMsr0bWSiwhyvqXyVyNa</t>
+  </si>
+  <si>
+    <t>bcit ( Computer Science and IT)</t>
+  </si>
+  <si>
+    <t>CT-26152</t>
+  </si>
+  <si>
+    <t>taniaanwer13@gmail.com</t>
+  </si>
+  <si>
+    <t>Tania Anwer</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1M-XxRNTh-F0TsuGLw3CxiWVJVQou3KUU</t>
+  </si>
+  <si>
+    <t>Electrical engineering</t>
+  </si>
+  <si>
+    <t>EE-165</t>
+  </si>
+  <si>
+    <t>muneebahmedd008@gmail.com</t>
+  </si>
+  <si>
+    <t>Muneeb Ahmed Shaikh</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1quexrz9P56n6XP4MzAbBUbmWXMaF2Urk</t>
+  </si>
+  <si>
+    <t>Electrical Engineering</t>
+  </si>
+  <si>
+    <t>arzoomakhdoom15@gmail.com</t>
+  </si>
+  <si>
+    <t>Arzoo Fatima</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1hxcIabDddt7JdcwrIrf8RWFX3tr9YxTs</t>
+  </si>
+  <si>
+    <t>EMD</t>
+  </si>
+  <si>
+    <t>NED</t>
+  </si>
+  <si>
+    <t>muhammadanas24190@gmail.com</t>
+  </si>
+  <si>
+    <t>Muhammad Anas</t>
+  </si>
+  <si>
+    <t>‪+92 325 7623295‬</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1rxHULx8A_1K0OF8pfYQNeycXKaEvveRn</t>
+  </si>
+  <si>
+    <t>CSIT</t>
+  </si>
+  <si>
+    <t>CT-26150</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
-  </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -149,19 +154,44 @@
     <font>
       <u/>
       <sz val="10"/>
-      <color rgb="FF0000FF"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
       <name val="Roboto"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F9FA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -169,51 +199,279 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF442F65"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF8F9FA"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFF8F9FA"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF8F9FA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF8F9FA"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFF8F9FA"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF8F9FA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF442F65"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFF8F9FA"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF8F9FA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF442F65"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF8F9FA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF8F9FA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF442F65"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF8F9FA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF442F65"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF8F9FA"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF8F9FA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF8F9FA"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF8F9FA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF442F65"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF442F65"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF442F65"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF8F9FA"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFF8F9FA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF8F9FA"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFF8F9FA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="22" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="3" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF5B3F86"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF5B3F86"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF5B3F86"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF5B3F86"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -238,13 +496,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF5B3F86"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF5B3F86"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF5B3F86"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF5B3F86"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Form Responses 1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -263,7 +537,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:I5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:I6">
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Timestamp"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Email Address"/>
@@ -492,7 +766,7 @@
     <col min="10" max="15" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -503,13 +777,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="6" t="s">
-        <v>31</v>
+      <c r="F1" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
@@ -521,111 +795,143 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
-        <v>46309.695078159726</v>
-      </c>
-      <c r="B2" s="3" t="s">
+    <row r="2" spans="1:9" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>46309.754259259258</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="4">
+        <v>3178321201</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="G2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="I2" s="6"/>
+    </row>
+    <row r="3" spans="1:9" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
+        <v>46309.761273148149</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="3" t="s">
+      <c r="C3" s="8" t="s">
         <v>16</v>
       </c>
+      <c r="D3" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="8">
+        <v>3306661534</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="10"/>
     </row>
-    <row r="3" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
-        <v>46309.707129467592</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="5" t="s">
+    <row r="4" spans="1:9" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11">
+        <v>46309.766921296294</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="3" t="s">
+      <c r="C4" s="12" t="s">
         <v>21</v>
       </c>
+      <c r="D4" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="12">
+        <v>3316713255</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="14"/>
     </row>
-    <row r="4" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
-        <v>46309.720478356481</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="3" t="s">
+    <row r="5" spans="1:9" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="15">
+        <v>46309.780949074076</v>
+      </c>
+      <c r="B5" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="C5" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="D5" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="16">
+        <v>3001568665</v>
+      </c>
+      <c r="F5" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G5" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="3">
-        <v>26037</v>
+      <c r="H5" s="18">
+        <v>2500</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
-        <v>46309.73021908565</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="5" t="s">
+    <row r="6" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="20">
+        <v>46309.79755787037</v>
+      </c>
+      <c r="B6" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>10</v>
-      </c>
+      <c r="C6" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="23"/>
     </row>
-    <row r="6" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="7" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="8" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="9" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -676,14 +982,15 @@
     <row r="54" ht="22.5" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="F5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{786C083C-D6D3-423E-8779-04A924B699F1}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{50760749-9FAA-4071-B749-86EFF38C15CF}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{6838B0F2-4B2C-459C-BF8E-8F6CD857AE5A}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{B04CF2C1-1EEF-4857-B6D2-035D6FF1273F}"/>
+    <hyperlink ref="F6" r:id="rId5" xr:uid="{2D114DDC-F59F-468E-94A1-A3BC51AE8857}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Upload all social images to Cloudinary and update DB records to permanent Cloudinary URLs
</commit_message>
<xml_diff>
--- a/assets/Qawalli.xlsx
+++ b/assets/Qawalli.xlsx
@@ -29,8 +29,9 @@
   </si>
   <si>
     <t>Attach screen shot of payment 
-Rs 500 normal 
-Rs 300 Participant
+Rs 500 Early Bird Discount
+Rs 500 Normal Pass
+Rs 300 The Engineer's Code Participant Pass
 Title: NEDUET CONTROLLER STUDENT AFFAIRS
 Account Number: 6-99-72-29314-714-262131
 IBAN: PK73MPBL9972477140262131
@@ -1221,7 +1222,7 @@
     <tableColumn name="Name" id="3"/>
     <tableColumn name="email address" id="4"/>
     <tableColumn name="Phone number" id="5"/>
-    <tableColumn name="Attach screen shot of payment _x000a_Rs 500 normal _x000a_Rs 300 Participant_x000a_Title: NEDUET CONTROLLER STUDENT AFFAIRS_x000a_Account Number: 6-99-72-29314-714-262131_x000a_IBAN: PK73MPBL9972477140262131_x000a_Bank Name: Habib Metropolitan Bank Limited_x000a_Bank Address: University Road Branch, Karachi_x000a_Branch Code: 50    _x000a_Swift Code: MPBLPKKA050" id="6"/>
+    <tableColumn name="Attach screen shot of payment _x000a_Rs 500 Early Bird Discount_x000a_Rs 500 Normal Pass_x000a_Rs 300 The Engineer's Code Participant Pass_x000a_Title: NEDUET CONTROLLER STUDENT AFFAIRS_x000a_Account Number: 6-99-72-29314-714-262131_x000a_IBAN: PK73MPBL9972477140262131_x000a_Bank Name: Habib Metropolitan Bank Limited_x000a_Bank Address: University Road Branch, Karachi_x000a_Branch Code: 50    _x000a_Swift Code: MPBLPKKA050" id="6"/>
     <tableColumn name="Department" id="7"/>
     <tableColumn name="Roll no" id="8"/>
     <tableColumn name="University" id="9"/>

</xml_diff>

<commit_message>
Sync Qawalli registrations - 2 new entries
</commit_message>
<xml_diff>
--- a/assets/Qawalli.xlsx
+++ b/assets/Qawalli.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="375">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1092,6 +1092,60 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1r_GoembZwAEIW6cM1NksYj0OiZcDe6Ri</t>
+  </si>
+  <si>
+    <t>mohsinaliraza767@gmail.com</t>
+  </si>
+  <si>
+    <t>Mohsin Ali Raza</t>
+  </si>
+  <si>
+    <t>03202251158</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1hcoBjgD_T6IGELIEomrJb_KJ7JfOGSgp</t>
+  </si>
+  <si>
+    <t>Computational Finance</t>
+  </si>
+  <si>
+    <t>CF-26050</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1q6zPz93LpiSqbAWkdvz2R63zS4VYyCP9</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1jcSBgMK6KlStl9WhtfRh7m14lFNhP0WX</t>
+  </si>
+  <si>
+    <t>hooriazai2.0@gmail.com</t>
+  </si>
+  <si>
+    <t>Hooria zai</t>
+  </si>
+  <si>
+    <t>Hooriazai2.0@gmail.com</t>
+  </si>
+  <si>
+    <t>03312132524</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1nnVn3YG3IYwI4txIvlJLwXEnZeUfQg9e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Textile sciences </t>
+  </si>
+  <si>
+    <t>Ts-23063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ned university </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1gnLfXYx3Dj_HzGacFBk_Jnj8mrBXJ1Oz</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=12QqfBpCtV7TgWfks2CMn7tWZzDNbZTFh</t>
   </si>
 </sst>
 </file>
@@ -1257,7 +1311,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:L62" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:L64" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="12">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Email Address" id="2"/>
@@ -3183,6 +3237,76 @@
         <v>356</v>
       </c>
     </row>
+    <row r="63" ht="22.5" customHeight="1">
+      <c r="A63" s="8">
+        <v>46309.95319920139</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="C63" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="D63" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="E63" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="F63" s="11" t="s">
+        <v>360</v>
+      </c>
+      <c r="G63" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="H63" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="I63" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="J63" s="11" t="s">
+        <v>363</v>
+      </c>
+      <c r="K63" s="11" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="64" ht="22.5" customHeight="1">
+      <c r="A64" s="8">
+        <v>46309.96783887732</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="E64" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="F64" s="11" t="s">
+        <v>369</v>
+      </c>
+      <c r="G64" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="H64" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="I64" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="J64" s="11" t="s">
+        <v>373</v>
+      </c>
+      <c r="K64" s="11" t="s">
+        <v>374</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="F2"/>
@@ -3252,10 +3376,16 @@
     <hyperlink r:id="rId65" ref="F62"/>
     <hyperlink r:id="rId66" ref="J62"/>
     <hyperlink r:id="rId67" ref="K62"/>
+    <hyperlink r:id="rId68" ref="F63"/>
+    <hyperlink r:id="rId69" ref="J63"/>
+    <hyperlink r:id="rId70" ref="K63"/>
+    <hyperlink r:id="rId71" ref="F64"/>
+    <hyperlink r:id="rId72" ref="J64"/>
+    <hyperlink r:id="rId73" ref="K64"/>
   </hyperlinks>
-  <drawing r:id="rId68"/>
+  <drawing r:id="rId74"/>
   <tableParts count="1">
-    <tablePart r:id="rId70"/>
+    <tablePart r:id="rId76"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Qawalli registrations - 1 new entries
</commit_message>
<xml_diff>
--- a/assets/Qawalli.xlsx
+++ b/assets/Qawalli.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="385">
   <si>
     <t>Timestamp</t>
   </si>
@@ -29,8 +29,7 @@
   </si>
   <si>
     <t>Attach screen shot of payment 
-Rs 500 Early Bird Discount
-Rs 500 Normal Pass
+Rs 700 Normal Pass
 Rs 300 The Engineer's Code Participant Pass
 Title: NEDUET CONTROLLER STUDENT AFFAIRS
 Account Number: 6-99-72-29314-714-262131
@@ -1146,6 +1145,36 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=12QqfBpCtV7TgWfks2CMn7tWZzDNbZTFh</t>
+  </si>
+  <si>
+    <t>shayaankhan1277@gmail.com</t>
+  </si>
+  <si>
+    <t>Shayan khan</t>
+  </si>
+  <si>
+    <t>Shayaankhan1277@gmail.com</t>
+  </si>
+  <si>
+    <t>03703488815</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=19Omtjla9k04ICYSZDysIbtVtQWbmx8Ht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materials Engineering </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MM-25019 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NED UNIVERSITY ENGINEERING AND TECHNOLOGY </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=19PHEZGO-FEOhLDcdA95_1wdSDbIaAWo5</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1lFuz2aJFKD8tUuXcBXkL5xzuh10F5sDA</t>
   </si>
 </sst>
 </file>
@@ -1311,14 +1340,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:L64" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:L65" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="12">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Email Address" id="2"/>
     <tableColumn name="Name" id="3"/>
     <tableColumn name="email address" id="4"/>
     <tableColumn name="Phone number" id="5"/>
-    <tableColumn name="Attach screen shot of payment _x000a_Rs 500 Early Bird Discount_x000a_Rs 500 Normal Pass_x000a_Rs 300 The Engineer's Code Participant Pass_x000a_Title: NEDUET CONTROLLER STUDENT AFFAIRS_x000a_Account Number: 6-99-72-29314-714-262131_x000a_IBAN: PK73MPBL9972477140262131_x000a_Bank Name: Habib Metropolitan Bank Limited_x000a_Bank Address: University Road Branch, Karachi_x000a_Branch Code: 50    _x000a_Swift Code: MPBLPKKA050" id="6"/>
+    <tableColumn name="Attach screen shot of payment _x000a_Rs 700 Normal Pass_x000a_Rs 300 The Engineer's Code Participant Pass_x000a_Title: NEDUET CONTROLLER STUDENT AFFAIRS_x000a_Account Number: 6-99-72-29314-714-262131_x000a_IBAN: PK73MPBL9972477140262131_x000a_Bank Name: Habib Metropolitan Bank Limited_x000a_Bank Address: University Road Branch, Karachi_x000a_Branch Code: 50    _x000a_Swift Code: MPBLPKKA050" id="6"/>
     <tableColumn name="Department" id="7"/>
     <tableColumn name="Roll no" id="8"/>
     <tableColumn name="University" id="9"/>
@@ -3307,6 +3336,41 @@
         <v>374</v>
       </c>
     </row>
+    <row r="65" ht="22.5" customHeight="1">
+      <c r="A65" s="8">
+        <v>46310.05200358796</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>375</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>376</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="E65" s="10" t="s">
+        <v>378</v>
+      </c>
+      <c r="F65" s="11" t="s">
+        <v>379</v>
+      </c>
+      <c r="G65" s="9" t="s">
+        <v>380</v>
+      </c>
+      <c r="H65" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="I65" s="9" t="s">
+        <v>382</v>
+      </c>
+      <c r="J65" s="11" t="s">
+        <v>383</v>
+      </c>
+      <c r="K65" s="11" t="s">
+        <v>384</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="F2"/>
@@ -3382,10 +3446,13 @@
     <hyperlink r:id="rId71" ref="F64"/>
     <hyperlink r:id="rId72" ref="J64"/>
     <hyperlink r:id="rId73" ref="K64"/>
+    <hyperlink r:id="rId74" ref="F65"/>
+    <hyperlink r:id="rId75" ref="J65"/>
+    <hyperlink r:id="rId76" ref="K65"/>
   </hyperlinks>
-  <drawing r:id="rId74"/>
+  <drawing r:id="rId77"/>
   <tableParts count="1">
-    <tablePart r:id="rId76"/>
+    <tablePart r:id="rId79"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>